<commit_message>
Added new test cases for VPOC and Multibill
</commit_message>
<xml_diff>
--- a/KatalonData/MultibillTestData/MultibillCCData.xlsx
+++ b/KatalonData/MultibillTestData/MultibillCCData.xlsx
@@ -1,38 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t465179\Documents\git\VPS-Katalon\VPS-Katalon\KatalonData\MultibillTestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr documentId="13_ncr:1_{AA39726B-62B3-4FCF-BBA2-CEB1EAB08D28}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41B68A5-7E06-4AF2-8129-8D8D498632B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="1" windowHeight="13097" windowWidth="24686" xWindow="3394" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" yWindow="3394"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" firstSheet="16" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="CCData" r:id="rId1" sheetId="1"/>
-    <sheet name="VerifySearchResult" r:id="rId2" sheetId="2"/>
-    <sheet name="VerifyAmountTextBoxEditable" r:id="rId3" sheetId="3"/>
-    <sheet name="VerifyNoModifyAmountandRedacted" r:id="rId4" sheetId="4"/>
-    <sheet name="VerifyALTIDRedacted" r:id="rId5" sheetId="5"/>
-    <sheet name="VerifyALTIDNotRedacted" r:id="rId6" sheetId="6"/>
-    <sheet name="VerifyMultipleBillFileAtSearch" r:id="rId7" sheetId="7"/>
-    <sheet name="VerifyStaticTextOnSearch" r:id="rId8" sheetId="8"/>
-    <sheet name="Verify2Pages" r:id="rId9" sheetId="9"/>
-    <sheet name="VerifyErroron2CharSearch" r:id="rId10" sheetId="10"/>
-    <sheet name="VerifyCANSearch" r:id="rId11" sheetId="11"/>
-    <sheet name="VerifyStreetAddressSearch" r:id="rId12" sheetId="12"/>
-    <sheet name="VerifyStaticTextOnViewCart" r:id="rId13" sheetId="13"/>
-    <sheet name="VerifyLookup1Search" r:id="rId14" sheetId="14"/>
-    <sheet name="VerifyUDF3Saerch" r:id="rId15" sheetId="15"/>
-    <sheet name="VerifyRemoveCartContent" r:id="rId16" sheetId="16"/>
-    <sheet name="VerifyDataOnCartContent" r:id="rId17" sheetId="17"/>
-    <sheet name="VerifyPaymentEntryPageCC" r:id="rId18" sheetId="18"/>
-    <sheet name="VerifyPaymentEntryPagePC" r:id="rId19" sheetId="19"/>
-    <sheet name="VerifyPaymentEntryPageCorp" r:id="rId20" sheetId="20"/>
+    <sheet name="CCData" sheetId="1" r:id="rId1"/>
+    <sheet name="VerifySearchResult" sheetId="2" r:id="rId2"/>
+    <sheet name="VerifyAmountTextBoxEditable" sheetId="3" r:id="rId3"/>
+    <sheet name="VerifyNoModifyAmountandRedacted" sheetId="4" r:id="rId4"/>
+    <sheet name="VerifyALTIDRedacted" sheetId="5" r:id="rId5"/>
+    <sheet name="VerifyALTIDNotRedacted" sheetId="6" r:id="rId6"/>
+    <sheet name="VerifyMultipleBillFileAtSearch" sheetId="7" r:id="rId7"/>
+    <sheet name="VerifyStaticTextOnSearch" sheetId="8" r:id="rId8"/>
+    <sheet name="Verify2Pages" sheetId="9" r:id="rId9"/>
+    <sheet name="VerifyErroron2CharSearch" sheetId="10" r:id="rId10"/>
+    <sheet name="VerifyCANSearch" sheetId="11" r:id="rId11"/>
+    <sheet name="VerifyStreetAddressSearch" sheetId="12" r:id="rId12"/>
+    <sheet name="VerifyStaticTextOnViewCart" sheetId="13" r:id="rId13"/>
+    <sheet name="VerifyLookup1Search" sheetId="14" r:id="rId14"/>
+    <sheet name="VerifyUDF3Saerch" sheetId="15" r:id="rId15"/>
+    <sheet name="VerifyRemoveCartContent" sheetId="16" r:id="rId16"/>
+    <sheet name="VerifyDataOnCartContent" sheetId="17" r:id="rId17"/>
+    <sheet name="VerifyPaymentEntryPageCC" sheetId="18" r:id="rId18"/>
+    <sheet name="VerifyPaymentEntryPagePC" sheetId="19" r:id="rId19"/>
+    <sheet name="VerifyPaymentEntryPageCorp" sheetId="20" r:id="rId20"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="162">
   <si>
     <t>Result</t>
   </si>
@@ -406,534 +406,9 @@
     <t>Fri Nov 21 13:46:58 EST 2025</t>
   </si>
   <si>
-    <t>Wed Dec 10 19:18:22 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:18:41 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:19:05 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:20:14 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:20:54 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:21:08 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:22:15 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:22:46 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:24:20 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:25:17 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:26:12 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:26:46 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:27:20 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:27:55 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:28:19 EST 2025</t>
-  </si>
-  <si>
-    <t>DECEMBER 31 ,2021</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 19:58:34 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 20:00:25 EST 2025</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Wed Dec 10 20:05:50 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 20:06:42 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 20:07:24 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 20:29:35 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 20:30:26 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Dec 10 20:30:58 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:46:54 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:47:25 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:51:05 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:51:24 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:51:50 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:51:59 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:52:35 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:53:00 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:53:36 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:53:53 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:54:50 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:55:00 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:55:32 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:57:04 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:58:00 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:58:56 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 14:59:31 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 15:00:05 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 15:00:40 EST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 15:01:05 EST 2025</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:48:07 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:48:25 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:48:49 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:48:57 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:49:34 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:49:59 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:50:34 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:50:48 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:51:46 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:51:56 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:52:28 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:54:02 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:55:00 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:55:55 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:56:29 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:57:04 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:57:39 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jan 30 12:58:04 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 09 13:26:57 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:08:39 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:08:57 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:09:23 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:09:32 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:10:08 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:10:32 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:11:21 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:12:18 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:12:28 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:13:01 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:14:40 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:15:36 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:16:31 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:17:05 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:17:40 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:18:14 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:18:41 EST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 11 21:49:08 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:53:36 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:53:55 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:54:19 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:54:29 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:55:05 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:55:30 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:56:03 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:56:18 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:57:14 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:57:24 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:57:56 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 15:59:27 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 16:00:24 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 16:01:19 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 16:01:54 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 16:02:29 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 16:03:04 EST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 12 16:03:29 EST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 14 21:19:25 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:32:19 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:32:37 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:33:01 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:33:10 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:33:47 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:34:16 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:34:51 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:35:05 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:36:01 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:36:10 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:36:48 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:38:17 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:39:13 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:40:07 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:40:42 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:41:16 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:41:50 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 16 22:42:15 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:33:59 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:34:17 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:34:44 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:34:52 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:35:34 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:35:58 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:36:32 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:36:46 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:37:51 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:38:01 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:38:32 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:40:02 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:40:58 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:41:52 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:42:26 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:43:01 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:43:35 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 17:43:59 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:38:17 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:38:37 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:39:05 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:39:46 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:41:06 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:42:03 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:43:11 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:43:57 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:45:27 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:45:37 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:49:31 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 21:53:18 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 22:01:15 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 22:01:50 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 22:03:30 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 22:04:36 EST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 27 22:05:01 EST 2026</t>
-  </si>
-  <si>
-    <t>Mon Mar 09 11:34:56 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:10:30 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:13:33 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:14:16 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:19:46 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:22:20 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:24:15 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:25:12 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:26:10 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:26:49 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:27:27 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:29:20 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:32:42 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:39:55 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:42:59 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 18:43:34 EDT 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 11 19:11:09 EDT 2026</t>
-  </si>
-  <si>
-    <t>Thu Mar 12 10:35:47 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Jul 17 12:55:08 EDT 2026</t>
-  </si>
-  <si>
-    <t>Fri Jul 17 13:24:17 EDT 2026</t>
-  </si>
-  <si>
     <t>Fri Jul 17 14:44:46 EDT 2026</t>
   </si>
   <si>
-    <t>Fri Jul 17 14:45:14 EDT 2026</t>
-  </si>
-  <si>
     <t>Fri Jul 17 14:45:46 EDT 2026</t>
   </si>
   <si>
@@ -980,6 +455,81 @@
   </si>
   <si>
     <t>Fri Jul 17 15:36:56 EDT 2026</t>
+  </si>
+  <si>
+    <t>DECEMBER 31 ,2029</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:18:10 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:18:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:18:31 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:19:09 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:19:19 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:20:00 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:21:07 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:21:53 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:23:19 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:23:28 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:23:59 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:25:08 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:25:54 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:26:39 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:27:12 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:27:45 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:28:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:28:41 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:47:13 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 21:51:17 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 22:00:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 22:20:10 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 22:27:40 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Sep 18 22:29:43 EDT 2026</t>
   </si>
 </sst>
 </file>
@@ -1092,49 +642,49 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="16">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="2" fillId="0" fontId="0" numFmtId="49" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="3" fillId="0" fontId="0" numFmtId="49" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
-    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0"/>
-    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="49" xfId="0"/>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="2" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0">
-      <alignment horizontal="left" indent="1" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyFont="1" borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0"/>
-    <xf applyBorder="1" applyFont="1" borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0"/>
-    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1151,10 +701,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -1189,7 +739,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin panose="020F0302020204030204" typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1224,7 +774,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin panose="020F0502020204030204" typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1318,21 +868,21 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="6350">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="12700">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="19050">
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1349,7 +899,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw algn="ctr" blurRad="57150" dir="5400000" dist="19050" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1401,18 +951,18 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" name="Office Theme" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:26" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1492,7 +1042,7 @@
         <v>24</v>
       </c>
     </row>
-    <row ht="72.900000000000006" r="2" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:26" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C2" s="1" t="s">
         <v>25</v>
       </c>
@@ -1563,7 +1113,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -1571,15 +1121,15 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A8BF27D-9E5B-43D3-A8C6-55BD0B2E602C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A8BF27D-9E5B-43D3-A8C6-55BD0B2E602C}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="24.4609375" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" width="15.07421875" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="24.46484375" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" width="15.06640625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1597,7 +1147,7 @@
       </c>
       <c r="F1" s="3"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
         <v>26</v>
@@ -1607,20 +1157,20 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71D7CF63-52CE-45A5-AAAD-49E5406A5D05}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71D7CF63-52CE-45A5-AAAD-49E5406A5D05}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.4609375" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.15234375" collapsed="true"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.46484375" collapsed="true"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.1328125" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1652,12 +1202,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="43.75" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>299</v>
+        <v>142</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -1673,7 +1223,7 @@
         <v>88</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I2" s="5">
         <v>13.03</v>
@@ -1682,7 +1232,7 @@
         <v>684958</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
@@ -1712,16 +1262,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176BCD28-A901-4577-AC2B-4D8F84F5F4AB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176BCD28-A901-4577-AC2B-4D8F84F5F4AB}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1753,12 +1303,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="43.75" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>301</v>
+        <v>144</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -1774,7 +1324,7 @@
         <v>88</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I2" s="5">
         <v>13.03</v>
@@ -1784,16 +1334,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBAB8D87-1612-4A54-9789-20EBA3899496}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBAB8D87-1612-4A54-9789-20EBA3899496}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1810,12 +1360,12 @@
         <v>45</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>309</v>
+        <v>152</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -1825,12 +1375,12 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>310</v>
+        <v>153</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>26</v>
@@ -1840,16 +1390,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C795593-D462-4484-9AA4-88FCDAFE3571}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C795593-D462-4484-9AA4-88FCDAFE3571}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1881,12 +1431,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="43.75" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>300</v>
+        <v>143</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -1902,7 +1452,7 @@
         <v>88</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I2" s="5">
         <v>13.03</v>
@@ -1911,7 +1461,7 @@
         <v>684958</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
@@ -1941,16 +1491,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{922E2DF4-99DD-461B-8823-21A4F73EC265}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{922E2DF4-99DD-461B-8823-21A4F73EC265}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1982,12 +1532,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="58.3" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="57" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>302</v>
+        <v>145</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2003,7 +1553,7 @@
         <v>88</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I2" s="5">
         <v>13.03</v>
@@ -2013,21 +1563,21 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D2F5DCD-3C8F-4880-BB50-8902A2B8FCEA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D2F5DCD-3C8F-4880-BB50-8902A2B8FCEA}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="16.4609375" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.921875" collapsed="true"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="7.61328125" collapsed="true"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="16.46484375" collapsed="true"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.9296875" collapsed="true"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="7.59765625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2059,12 +1609,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>307</v>
+        <v>150</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2080,7 +1630,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15">
-        <v>44561</v>
+        <v>47483</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -2090,23 +1640,23 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97872C09-914A-48DE-8F4E-FDB918E9AE67}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97872C09-914A-48DE-8F4E-FDB918E9AE67}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="5.61328125" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.07421875" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="16.4609375" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.921875" collapsed="true"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="5.59765625" collapsed="true"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.06640625" collapsed="true"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="16.46484375" collapsed="true"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.9296875" collapsed="true"/>
     <col min="8" max="8" customWidth="true" width="22.0" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2138,12 +1688,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>298</v>
+        <v>141</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2159,7 +1709,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -2168,7 +1718,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s" s="0">
         <v>56</v>
       </c>
@@ -2183,16 +1733,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC5830D-66D0-4550-8001-686B3F1A766F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC5830D-66D0-4550-8001-686B3F1A766F}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2224,12 +1774,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>304</v>
+        <v>147</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2245,7 +1795,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15">
-        <v>44561</v>
+        <v>47483</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -2254,7 +1804,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
@@ -2269,16 +1819,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA84A4D-C922-4030-9CED-DABBEF75479D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA84A4D-C922-4030-9CED-DABBEF75479D}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2310,12 +1860,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>306</v>
+        <v>149</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2331,7 +1881,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15">
-        <v>44561</v>
+        <v>47483</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -2340,7 +1890,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
@@ -2355,23 +1905,23 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A683BE9-6249-421D-92CB-328DFD4DF946}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A683BE9-6249-421D-92CB-328DFD4DF946}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="25.921875" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="5.61328125" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.3828125" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.921875" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" style="7" width="9.15234375" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="25.9296875" collapsed="true"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="5.59765625" collapsed="true"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.3984375" collapsed="true"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.9296875" collapsed="true"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" style="7" width="9.1328125" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2403,12 +1953,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>308</v>
+        <v>151</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2424,7 +1974,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -2433,7 +1983,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
@@ -2463,16 +2013,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12B0A87-644D-4675-93A2-DC39D9AADE64}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12B0A87-644D-4675-93A2-DC39D9AADE64}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2504,12 +2054,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>305</v>
+        <v>148</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2525,7 +2075,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15">
-        <v>44561</v>
+        <v>47483</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -2534,7 +2084,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
@@ -2549,19 +2099,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{051F4528-1B41-4D78-BCA4-48AC174370CB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{051F4528-1B41-4D78-BCA4-48AC174370CB}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="25.921875" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="25.9296875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2593,12 +2143,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>297</v>
+        <v>161</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2614,7 +2164,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15">
-        <v>44561</v>
+        <v>47483</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -2623,7 +2173,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="5"/>
@@ -2633,19 +2183,19 @@
       <c r="J3" s="1"/>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{320D1D33-46D9-47A1-8D21-2F325C6EB804}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{320D1D33-46D9-47A1-8D21-2F325C6EB804}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.921875" collapsed="true"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.9296875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2677,7 +2227,7 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
@@ -2698,7 +2248,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15">
-        <v>44561</v>
+        <v>47483</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>117</v>
@@ -2707,25 +2257,25 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="H3" s="6" t="s">
         <v>55</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869053C2-BECE-477A-A52F-F9A660E766F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869053C2-BECE-477A-A52F-F9A660E766F1}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="25.921875" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="25.9296875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2757,12 +2307,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>296</v>
+        <v>139</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2778,7 +2328,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15">
-        <v>44561</v>
+        <v>47483</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -2788,28 +2338,28 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB854B13-0493-48E8-AA80-CD6F2F5005DA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB854B13-0493-48E8-AA80-CD6F2F5005DA}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.921875" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="25.921875" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="5.61328125" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="7.23046875" collapsed="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="5.9296875" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="25.9296875" collapsed="true"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="5.59765625" collapsed="true"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="7.19921875" collapsed="true"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="13.0" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="16.4609375" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="15.921875" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="8.07421875" collapsed="true"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="7.53515625" collapsed="true"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="13.921875" collapsed="true"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="16.46484375" collapsed="true"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="15.9296875" collapsed="true"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="8.06640625" collapsed="true"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="7.53125" collapsed="true"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="13.9296875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2841,12 +2391,12 @@
         <v>53</v>
       </c>
     </row>
-    <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>294</v>
+        <v>138</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2862,7 +2412,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15">
-        <v>44561</v>
+        <v>47483</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -2872,27 +2422,27 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36947155-855C-418A-BB46-98E870DFBFDC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36947155-855C-418A-BB46-98E870DFBFDC}">
   <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="25.61328125" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" width="12.84375" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="23.3828125" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="17.921875" collapsed="true"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="12.921875" collapsed="true"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="23.3828125" collapsed="true"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="17.921875" collapsed="true"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="17.53515625" collapsed="true"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="14.69140625" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="25.59765625" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" width="12.86328125" collapsed="true"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="23.3984375" collapsed="true"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="17.9296875" collapsed="true"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.9296875" collapsed="true"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="23.3984375" collapsed="true"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="17.9296875" collapsed="true"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="17.53125" collapsed="true"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="14.6640625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2948,7 +2498,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A2" s="5" t="s">
         <v>56</v>
       </c>
@@ -2969,7 +2519,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I2" s="8">
         <v>16.510000000000002</v>
@@ -3003,16 +2553,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E46036D-3E0A-4CA8-9437-AC70B02E484B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E46036D-3E0A-4CA8-9437-AC70B02E484B}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -3056,12 +2606,12 @@
         <v>81</v>
       </c>
     </row>
-    <row ht="113.15" r="2" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:15" ht="127.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>311</v>
+        <v>154</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -3102,19 +2652,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B0777A2-8D17-46EC-97AB-260FCB0FA79E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B0777A2-8D17-46EC-97AB-260FCB0FA79E}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="5.61328125" collapsed="true"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="5.59765625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row ht="29.15" r="1" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -3131,12 +2681,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>303</v>
+        <v>155</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -3146,7 +2696,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
@@ -3161,6 +2711,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>